<commit_message>
Made a lot of changes
</commit_message>
<xml_diff>
--- a/app/static/downloads/SESA_Student_Upload_Template.xlsx
+++ b/app/static/downloads/SESA_Student_Upload_Template.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>highschool</t>
+          <t>shs</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>highschool</t>
+          <t>shs</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>middleschool</t>
+          <t>shs</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>middleschool</t>
+          <t>shs</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>primaryschool</t>
+          <t>shs</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -1936,7 +1936,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>level         →  Must be exactly one of: primaryschool | middleschool | highschool | university</t>
+          <t>level         →  Must be exactly one of: jhs | shs | university</t>
         </is>
       </c>
     </row>

</xml_diff>